<commit_message>
Added instructions to templates
</commit_message>
<xml_diff>
--- a/templates/desiderata_template.xlsx
+++ b/templates/desiderata_template.xlsx
@@ -2,13 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\seria\Desktop\Repositories\shifter\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D5B14B1-6C92-44BD-AED2-3916AF3EDCD8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21372E65-CBBD-44F9-A28C-90AFD84E5358}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="26835" windowHeight="12060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>Persona</t>
   </si>
@@ -46,59 +41,38 @@
     <t>Tirocinio</t>
   </si>
   <si>
-    <t>Menoncello</t>
-  </si>
-  <si>
-    <t>Y</t>
-  </si>
-  <si>
-    <t>3/11/2025 P, 12/11/2025 P, 14/11/2025 M, 19/11/2025 P, 21/11/2025 P</t>
-  </si>
-  <si>
-    <t>01/11/2025, 29/11/2025</t>
-  </si>
-  <si>
-    <t>3/11/2025-7/11/2025,10/11/2025-14/11/2025,17/11/2025-21/11/2025,24/11/2025-28/11/2025</t>
-  </si>
-  <si>
-    <t>Messana</t>
-  </si>
-  <si>
-    <t>01/11/2025, 22/11/2025</t>
-  </si>
-  <si>
-    <t>Scardino</t>
-  </si>
-  <si>
-    <t>15/11/2025, 22/11/2025</t>
-  </si>
-  <si>
-    <t>Rudenko</t>
-  </si>
-  <si>
-    <t>Odales</t>
-  </si>
-  <si>
-    <t>1/11/2025, 15/11/2025</t>
-  </si>
-  <si>
-    <t>4/11/2025 P, 11/11/2025 P, 18/11/2025 P, 25/11/2025 P, 6/11/2025 MP</t>
-  </si>
-  <si>
-    <t>5/11/2025 P, 14/11/2025 P, 18/11/2025 P, 24/11/2025 P</t>
-  </si>
-  <si>
-    <t>3/11/2025 P, 7/11/2025 P, 20/11/2025 P, 25/11/2025 P</t>
-  </si>
-  <si>
-    <t>5/11/2025 P, 13/11/2025 P, 18/11/2025 P, 24/11/2025 P, 26/11/2025 P</t>
+    <t>nomepersona</t>
+  </si>
+  <si>
+    <t>Indicare un valore numerico intero: 0 - bassa priorita, &gt;0 - alta priorita</t>
+  </si>
+  <si>
+    <t>Indicare il sabato del weekend vietato; sintassi: GG/MM/YYYY</t>
+  </si>
+  <si>
+    <t>Indicare l'intervallo di date; sintassi: GG/MM/YYYY-GG/MM/YYYY; se data singola inserire comunque l'intervallo (e.g. 05/11/2025-05/11/2025)</t>
+  </si>
+  <si>
+    <t>Indicare l'intervallo di date di tirocinio. Se si intende lasciare disponibilità ai weekend per altri turni, indicare solamente i giorni lun-ven. (e.g. 3/11/2025-7/11/2025,10/11/2025-14/11/2025)</t>
+  </si>
+  <si>
+    <t>Indicare un valore numerico intero: 0 - bassa priorità, &gt;0 - alta priorità</t>
+  </si>
+  <si>
+    <t>Indicare disponibilità a turni notturni; disponibile: Y, non disponibile: N</t>
+  </si>
+  <si>
+    <t>Indicare la data seguita dal tipo di turno vietato; sintassi: GG/MM/YYYY MNP; si può inserire solo M, N, o P, oppure combinazioni di essi (e.g. MP, o NP); non inserire ulteriori caratteri (e.g. "01/01/2025 no P")</t>
+  </si>
+  <si>
+    <t>PRIMA DI COMPILARE RIMUOVERE LA RIGA 2 e 3. LASCIARE SOLAMENTE LA RIGA 1.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -233,8 +207,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="34">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -412,12 +392,6 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -583,7 +557,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -939,8 +913,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.5703125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -973,18 +950,21 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" t="s">
         <v>9</v>
       </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
       <c r="E2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" t="s">
         <v>10</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>11</v>
       </c>
       <c r="H2" t="s">
@@ -993,82 +973,14 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-      <c r="D6">
-        <v>1</v>
-      </c>
-      <c r="E6" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" t="s">
-        <v>19</v>
-      </c>
+      <c r="E5" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>